<commit_message>
Add new strategy comparison script and associated files for extended hours analysis
- Introduced `update_ndx_strategy_comparison_20261024.py` to extend the audited comparison and chart every active strategy without model fitting.
- Added new lock and tar files for the default bundle.
- Created a new LaTeX format file for the generated output.
- Implemented functions to load, prepare, and audit strategy data, ensuring integrity and correctness of metrics.
- Generated detailed output files including all strategies and extended hours accounts.
- Developed charts for visual representation of historical leaders and benchmarks.
- Updated methodology and documentation to reflect the latest analysis and findings.
</commit_message>
<xml_diff>
--- a/outputs/01a15702-86c3-7463-ae6c-24606895c7cf/strategy_comparison_20261020/NASDAQ100_strategy_comparison.xlsx
+++ b/outputs/01a15702-86c3-7463-ae6c-24606895c7cf/strategy_comparison_20261020/NASDAQ100_strategy_comparison.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Models" sheetId="1" r:id="R749fa8f2355c4e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defensive" sheetId="2" r:id="R6670b2e48680447a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio variants" sheetId="3" r:id="R3b605cdca6fb4f53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R4eac9d6588654333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Models" sheetId="1" r:id="R5b085ea21eb64f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defensive" sheetId="2" r:id="R282023bcd8704416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio variants" sheetId="3" r:id="R5a5d6249fd06448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="Ra2298c5e527c4709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended-hours" sheetId="5" r:id="Ra06df26a5d5242eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,10 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="0.000"/>
     <x:numFmt numFmtId="201" formatCode="0.00%"/>
     <x:numFmt numFmtId="202" formatCode="0.0000"/>
+    <x:numFmt numFmtId="203" formatCode="0&quot;x&quot;"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -56,12 +58,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF18344F"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -90,7 +97,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -155,6 +162,18 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -163,8 +182,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Comparison1" displayName="Comparison1" ref="A5:H69" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:H69"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Comparison1" displayName="Comparison1" ref="A5:H77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:H77"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Strategy"/>
     <x:tableColumn id="2" name="Study"/>
@@ -208,6 +227,25 @@
     <x:tableColumn id="6" name="Max drawdown"/>
     <x:tableColumn id="7" name="SR 95% lower"/>
     <x:tableColumn id="8" name="SR 95% upper"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ExtendedHoursAccounts" displayName="ExtendedHoursAccounts" ref="A5:J71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:J71"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="Strategy"/>
+    <x:tableColumn id="2" name="Role"/>
+    <x:tableColumn id="3" name="Seed"/>
+    <x:tableColumn id="4" name="Fee multiple"/>
+    <x:tableColumn id="5" name="Sharpe"/>
+    <x:tableColumn id="6" name="CAGR"/>
+    <x:tableColumn id="7" name="RankIC"/>
+    <x:tableColumn id="8" name="Max drawdown"/>
+    <x:tableColumn id="9" name="SR 95% lower"/>
+    <x:tableColumn id="10" name="SR 95% upper"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -445,7 +483,7 @@
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>2022–2025 • net base-cost returns • 3% Sharpe hurdle • 10,000 block resamples</x:v>
+        <x:v>2022–2025 • updated October 24 • base costs • 3% SR hurdle • 10,000 block resamples</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2155,10 +2193,218 @@
         <x:v>1.3987374592</x:v>
       </x:c>
     </x:row>
+    <x:row r="70" ht="23" customHeight="1">
+      <x:c r="A70" s="2" t="str">
+        <x:v>THINK + mixer / Daily / ten seeds</x:v>
+      </x:c>
+      <x:c r="B70" s="2" t="str">
+        <x:v>Extended-hours information</x:v>
+      </x:c>
+      <x:c r="C70" s="11" t="n">
+        <x:v>0.4964676002181367</x:v>
+      </x:c>
+      <x:c r="D70" s="12" t="n">
+        <x:v>0.14536329142518786</x:v>
+      </x:c>
+      <x:c r="E70" s="13" t="n">
+        <x:v>0.0048493578263471</x:v>
+      </x:c>
+      <x:c r="F70" s="12" t="n">
+        <x:v>-0.3711259939433199</x:v>
+      </x:c>
+      <x:c r="G70" s="11" t="n">
+        <x:v>-0.3316510050464303</x:v>
+      </x:c>
+      <x:c r="H70" s="11" t="n">
+        <x:v>1.3670552912857934</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="23" customHeight="1">
+      <x:c r="A71" s="2" t="str">
+        <x:v>THINK + mixer / Daily / new five seeds</x:v>
+      </x:c>
+      <x:c r="B71" s="2" t="str">
+        <x:v>Extended-hours information</x:v>
+      </x:c>
+      <x:c r="C71" s="11" t="n">
+        <x:v>0.5364645380064392</x:v>
+      </x:c>
+      <x:c r="D71" s="12" t="n">
+        <x:v>0.15506488269543164</x:v>
+      </x:c>
+      <x:c r="E71" s="13" t="n">
+        <x:v>0.0081765583185379</x:v>
+      </x:c>
+      <x:c r="F71" s="12" t="n">
+        <x:v>-0.3128163233905591</x:v>
+      </x:c>
+      <x:c r="G71" s="11" t="n">
+        <x:v>-0.3212700209602253</x:v>
+      </x:c>
+      <x:c r="H71" s="11" t="n">
+        <x:v>1.427256445191111</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="23" customHeight="1">
+      <x:c r="A72" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / ten seeds</x:v>
+      </x:c>
+      <x:c r="B72" s="2" t="str">
+        <x:v>Extended-hours information</x:v>
+      </x:c>
+      <x:c r="C72" s="11" t="n">
+        <x:v>0.4882238564367686</x:v>
+      </x:c>
+      <x:c r="D72" s="12" t="n">
+        <x:v>0.14226921456410785</x:v>
+      </x:c>
+      <x:c r="E72" s="13" t="n">
+        <x:v>0.0035727536866006</x:v>
+      </x:c>
+      <x:c r="F72" s="12" t="n">
+        <x:v>-0.4011704221619038</x:v>
+      </x:c>
+      <x:c r="G72" s="11" t="n">
+        <x:v>-0.3665240836934171</x:v>
+      </x:c>
+      <x:c r="H72" s="11" t="n">
+        <x:v>1.3827586125394058</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="23" customHeight="1">
+      <x:c r="A73" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / original five seeds</x:v>
+      </x:c>
+      <x:c r="B73" s="2" t="str">
+        <x:v>Extended-hours information</x:v>
+      </x:c>
+      <x:c r="C73" s="11" t="n">
+        <x:v>0.6024624994600978</x:v>
+      </x:c>
+      <x:c r="D73" s="12" t="n">
+        <x:v>0.1860236058844805</x:v>
+      </x:c>
+      <x:c r="E73" s="13" t="n">
+        <x:v>0.0063408707312977</x:v>
+      </x:c>
+      <x:c r="F73" s="12" t="n">
+        <x:v>-0.37161827435781014</x:v>
+      </x:c>
+      <x:c r="G73" s="11" t="n">
+        <x:v>-0.2193536466130756</x:v>
+      </x:c>
+      <x:c r="H73" s="11" t="n">
+        <x:v>1.4754691689101456</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="23" customHeight="1">
+      <x:c r="A74" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / new five seeds</x:v>
+      </x:c>
+      <x:c r="B74" s="2" t="str">
+        <x:v>Extended-hours information</x:v>
+      </x:c>
+      <x:c r="C74" s="11" t="n">
+        <x:v>0.47398709120623245</x:v>
+      </x:c>
+      <x:c r="D74" s="12" t="n">
+        <x:v>0.13432742993395266</x:v>
+      </x:c>
+      <x:c r="E74" s="13" t="n">
+        <x:v>0.0060933322472734</x:v>
+      </x:c>
+      <x:c r="F74" s="12" t="n">
+        <x:v>-0.33121069853341756</x:v>
+      </x:c>
+      <x:c r="G74" s="11" t="n">
+        <x:v>-0.386761700440253</x:v>
+      </x:c>
+      <x:c r="H74" s="11" t="n">
+        <x:v>1.381458473720616</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="23" customHeight="1">
+      <x:c r="A75" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / ten seeds</x:v>
+      </x:c>
+      <x:c r="B75" s="2" t="str">
+        <x:v>Extended-hours information</x:v>
+      </x:c>
+      <x:c r="C75" s="11" t="n">
+        <x:v>0.5191500032056338</x:v>
+      </x:c>
+      <x:c r="D75" s="12" t="n">
+        <x:v>0.15356400976834336</x:v>
+      </x:c>
+      <x:c r="E75" s="13" t="n">
+        <x:v>0.0037740295593641</x:v>
+      </x:c>
+      <x:c r="F75" s="12" t="n">
+        <x:v>-0.3832320310700549</x:v>
+      </x:c>
+      <x:c r="G75" s="11" t="n">
+        <x:v>-0.3452746799425182</x:v>
+      </x:c>
+      <x:c r="H75" s="11" t="n">
+        <x:v>1.425365964092924</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="23" customHeight="1">
+      <x:c r="A76" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / original five seeds</x:v>
+      </x:c>
+      <x:c r="B76" s="2" t="str">
+        <x:v>Extended-hours information</x:v>
+      </x:c>
+      <x:c r="C76" s="11" t="n">
+        <x:v>0.7002722836906295</x:v>
+      </x:c>
+      <x:c r="D76" s="12" t="n">
+        <x:v>0.22385598411825272</x:v>
+      </x:c>
+      <x:c r="E76" s="13" t="n">
+        <x:v>0.0060550276299253</x:v>
+      </x:c>
+      <x:c r="F76" s="12" t="n">
+        <x:v>-0.35013286984215053</x:v>
+      </x:c>
+      <x:c r="G76" s="11" t="n">
+        <x:v>-0.1393513711221214</x:v>
+      </x:c>
+      <x:c r="H76" s="11" t="n">
+        <x:v>1.5935183268359752</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="23" customHeight="1">
+      <x:c r="A77" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / new five seeds</x:v>
+      </x:c>
+      <x:c r="B77" s="2" t="str">
+        <x:v>Extended-hours information</x:v>
+      </x:c>
+      <x:c r="C77" s="11" t="n">
+        <x:v>0.4802168579045056</x:v>
+      </x:c>
+      <x:c r="D77" s="12" t="n">
+        <x:v>0.13693671292731538</x:v>
+      </x:c>
+      <x:c r="E77" s="13" t="n">
+        <x:v>0.0067411410003181</x:v>
+      </x:c>
+      <x:c r="F77" s="12" t="n">
+        <x:v>-0.34402710440142015</x:v>
+      </x:c>
+      <x:c r="G77" s="11" t="n">
+        <x:v>-0.3816345022820374</x:v>
+      </x:c>
+      <x:c r="H77" s="11" t="n">
+        <x:v>1.3651643080407354</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0d5c78954e5462f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra43f46b7a2b8413c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3111,7 +3357,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf7870df2e8a4117"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf21820dc35f7456d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7730,7 +7976,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f1be1ee4f294a5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75378111187d4611"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7785,7 +8031,7 @@
         <x:v>Financial metrics</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>Net returns at each study’s base modeled trading costs. Ensemble forecasts; no seed selected by test performance.</x:v>
+        <x:v>Net returns at base modeled costs in the first three tabs. The Extended-hours tab also discloses individual seeds and 2x/4x fee stresses.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52" customHeight="1">
@@ -7873,7 +8119,7 @@
         <x:v>Excluded repetitions</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>Reference aliases, individual seeds, fee stresses and seed-bootstrap accounts are omitted. Distinct declared selection policies remain, even when their realized paths coincide.</x:v>
+        <x:v>Main tabs omit reference aliases, individual seeds, fee stresses and seed-bootstrap accounts. All 66 extended-hours accounts are separately disclosed. Original-five daily and the three base-cost benchmarks reuse existing main-table rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="52" customHeight="1">
@@ -7913,7 +8159,7 @@
         <x:v>Source studies</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
-        <x:v>Audited original monthly/top-k/long-short, matched Alpaca, ranking, broad-feature, frozen-core correction and seed-expansion studies.</x:v>
+        <x:v>Audited original monthly/top-k/long-short, matched Alpaca, ranking, broad-feature, frozen-core correction and seed-expansion studies. Extended-hours and premarket information study (October 24) is included.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="52" customHeight="1">
@@ -7932,7 +8178,2278 @@
         <x:v>Andrew W. Lo, The Statistics of Sharpe Ratios (2002): https://alo.mit.edu/publications/page/18/</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="52" customHeight="1">
+      <x:c r="A26" s="25" t="str">
+        <x:v>Extended-hours clock</x:v>
+      </x:c>
+      <x:c r="B26" s="24" t="str">
+        <x:v>AH: prior regular close through 20:00 ET. PM: next exchange session 04:00–09:15 ET. All views decide at 09:20 ET and fill at that session’s regular close.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="52" customHeight="1">
+      <x:c r="A27" s="25" t="str">
+        <x:v>Extended-hours seeds</x:v>
+      </x:c>
+      <x:c r="B27" s="24" t="str">
+        <x:v>Primary ten seeds are fixed before metrics. Original-five and new-five ensembles and all individual seeds are diagnostics. The original five daily forecasts reproduce the earlier model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="52" customHeight="1">
+      <x:c r="A28" s="25" t="str">
+        <x:v>Extended-hours limits</x:v>
+      </x:c>
+      <x:c r="B28" s="24" t="str">
+        <x:v>About 50% of member sessions have at least four AH bars and 46% have at least four PM bars. Missing activity is flagged. PM prior-close price gaps were excluded to avoid raw corporate-action discontinuities.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="52" customHeight="1">
+      <x:c r="A29" s="25" t="str">
+        <x:v>Current leaders</x:v>
+      </x:c>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Highest base-cost CAGR: StockMixer top 5. Highest base-cost Sharpe: StockMixer top 5, 75% long / 25% short. Highest standard top-10 ensemble CAGR: original-five THINK + mixer with AH + PM. These are historical rankings, not forward selection rules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="52" customHeight="1">
+      <x:c r="A30" s="25" t="str">
+        <x:v>Seed evidence</x:v>
+      </x:c>
+      <x:c r="B30" s="24" t="str">
+        <x:v>AH + PM improved 5/10 individual seeds. Its original-five CAGR rose from 19.60% to 22.39%, but the new-five group fell from 15.51% to 13.69%. Primary paired intervals include zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="52" customHeight="1">
+      <x:c r="A31" s="25" t="str">
+        <x:v>Sources and charts</x:v>
+      </x:c>
+      <x:c r="B31" s="24" t="str">
+        <x:v>See root charts.md for every main strategy and all additional extended-hours seed/cost accounts, source report links and paired uncertainty. Updated analysis: update_ndx_strategy_comparison_20261024.py.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF456582"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="66" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="23" customHeight="1">
+      <x:c r="A1" s="2"/>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+    </x:row>
+    <x:row r="2" ht="23" customHeight="1">
+      <x:c r="A2" s="4" t="str">
+        <x:v>Extended-hours accounts and sensitivities</x:v>
+      </x:c>
+      <x:c r="B2" s="5"/>
+      <x:c r="C2" s="5"/>
+      <x:c r="D2" s="5"/>
+      <x:c r="E2" s="5"/>
+      <x:c r="F2" s="5"/>
+      <x:c r="G2" s="5"/>
+      <x:c r="H2" s="5"/>
+      <x:c r="I2" s="5"/>
+      <x:c r="J2" s="5"/>
+    </x:row>
+    <x:row r="3" ht="23" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>2022–2025 • all 66 accounts • fixed primary ten seeds; other groups diagnostic • 20-session SR intervals</x:v>
+      </x:c>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+      <x:c r="H3" s="2"/>
+      <x:c r="I3" s="2"/>
+      <x:c r="J3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="23" customHeight="1">
+      <x:c r="A4" s="2"/>
+      <x:c r="B4" s="2"/>
+      <x:c r="C4" s="2"/>
+      <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
+      <x:c r="F4" s="2"/>
+      <x:c r="G4" s="2"/>
+      <x:c r="H4" s="2"/>
+      <x:c r="I4" s="2"/>
+      <x:c r="J4" s="2"/>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="28" t="str">
+        <x:v>Strategy</x:v>
+      </x:c>
+      <x:c r="B5" s="28" t="str">
+        <x:v>Role</x:v>
+      </x:c>
+      <x:c r="C5" s="28" t="str">
+        <x:v>Seed</x:v>
+      </x:c>
+      <x:c r="D5" s="28" t="str">
+        <x:v>Fee multiple</x:v>
+      </x:c>
+      <x:c r="E5" s="28" t="str">
+        <x:v>Sharpe</x:v>
+      </x:c>
+      <x:c r="F5" s="28" t="str">
+        <x:v>CAGR</x:v>
+      </x:c>
+      <x:c r="G5" s="28" t="str">
+        <x:v>RankIC</x:v>
+      </x:c>
+      <x:c r="H5" s="28" t="str">
+        <x:v>Max drawdown</x:v>
+      </x:c>
+      <x:c r="I5" s="28" t="str">
+        <x:v>SR 95% lower</x:v>
+      </x:c>
+      <x:c r="J5" s="28" t="str">
+        <x:v>SR 95% upper</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="23" customHeight="1">
+      <x:c r="A6" s="2" t="str">
+        <x:v>THINK + mixer / Daily / ten seeds</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>Primary ten-seed ensemble</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D6" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="n">
+        <x:v>0.4964676002181367</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="n">
+        <x:v>0.14536329142518786</x:v>
+      </x:c>
+      <x:c r="G6" s="13" t="n">
+        <x:v>0.0048493578263471</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="n">
+        <x:v>-0.3711259939433199</x:v>
+      </x:c>
+      <x:c r="I6" s="11" t="n">
+        <x:v>-0.3316510050464303</x:v>
+      </x:c>
+      <x:c r="J6" s="11" t="n">
+        <x:v>1.3670552912857934</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="23" customHeight="1">
+      <x:c r="A7" s="2" t="str">
+        <x:v>THINK + mixer / Daily / ten seeds</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D7" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="n">
+        <x:v>0.44526708898880385</x:v>
+      </x:c>
+      <x:c r="F7" s="12" t="n">
+        <x:v>0.12730214267892065</x:v>
+      </x:c>
+      <x:c r="G7" s="13" t="n">
+        <x:v>0.0048493578263471</x:v>
+      </x:c>
+      <x:c r="H7" s="12" t="n">
+        <x:v>-0.3800101876806803</x:v>
+      </x:c>
+      <x:c r="I7" s="11" t="n">
+        <x:v>-0.3802917642849086</x:v>
+      </x:c>
+      <x:c r="J7" s="11" t="n">
+        <x:v>1.3119880753802542</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="23" customHeight="1">
+      <x:c r="A8" s="2" t="str">
+        <x:v>THINK + mixer / Daily / ten seeds</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D8" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="n">
+        <x:v>0.3432223800435531</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="n">
+        <x:v>0.09210525945792693</x:v>
+      </x:c>
+      <x:c r="G8" s="13" t="n">
+        <x:v>0.0048493578263471</x:v>
+      </x:c>
+      <x:c r="H8" s="12" t="n">
+        <x:v>-0.3974358544683637</x:v>
+      </x:c>
+      <x:c r="I8" s="11" t="n">
+        <x:v>-0.4771917759142083</x:v>
+      </x:c>
+      <x:c r="J8" s="11" t="n">
+        <x:v>1.2059891593118874</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="23" customHeight="1">
+      <x:c r="A9" s="2" t="str">
+        <x:v>THINK + mixer / Daily / original five seeds</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>Seed-subgroup diagnostic</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D9" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="n">
+        <x:v>0.6290114470394799</x:v>
+      </x:c>
+      <x:c r="F9" s="12" t="n">
+        <x:v>0.19603725534403432</x:v>
+      </x:c>
+      <x:c r="G9" s="13" t="n">
+        <x:v>0.0074059162149529</x:v>
+      </x:c>
+      <x:c r="H9" s="12" t="n">
+        <x:v>-0.39444936012383425</x:v>
+      </x:c>
+      <x:c r="I9" s="11" t="n">
+        <x:v>-0.1864504227908077</x:v>
+      </x:c>
+      <x:c r="J9" s="11" t="n">
+        <x:v>1.504645018539174</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="23" customHeight="1">
+      <x:c r="A10" s="2" t="str">
+        <x:v>THINK + mixer / Daily / original five seeds</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D10" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="n">
+        <x:v>0.5721386112587606</x:v>
+      </x:c>
+      <x:c r="F10" s="12" t="n">
+        <x:v>0.17469917488077563</x:v>
+      </x:c>
+      <x:c r="G10" s="13" t="n">
+        <x:v>0.0074059162149529</x:v>
+      </x:c>
+      <x:c r="H10" s="12" t="n">
+        <x:v>-0.4038044623684286</x:v>
+      </x:c>
+      <x:c r="I10" s="11" t="n">
+        <x:v>-0.2385534817873527</x:v>
+      </x:c>
+      <x:c r="J10" s="11" t="n">
+        <x:v>1.4442437206669714</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="23" customHeight="1">
+      <x:c r="A11" s="2" t="str">
+        <x:v>THINK + mixer / Daily / original five seeds</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D11" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="n">
+        <x:v>0.45898659897020616</x:v>
+      </x:c>
+      <x:c r="F11" s="12" t="n">
+        <x:v>0.13330465436505703</x:v>
+      </x:c>
+      <x:c r="G11" s="13" t="n">
+        <x:v>0.0074059162149529</x:v>
+      </x:c>
+      <x:c r="H11" s="12" t="n">
+        <x:v>-0.4220372767018147</x:v>
+      </x:c>
+      <x:c r="I11" s="11" t="n">
+        <x:v>-0.3495219871890293</x:v>
+      </x:c>
+      <x:c r="J11" s="11" t="n">
+        <x:v>1.3304346547523611</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="23" customHeight="1">
+      <x:c r="A12" s="2" t="str">
+        <x:v>THINK + mixer / Daily / new five seeds</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="str">
+        <x:v>Seed-subgroup diagnostic</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D12" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="11" t="n">
+        <x:v>0.5364645380064392</x:v>
+      </x:c>
+      <x:c r="F12" s="12" t="n">
+        <x:v>0.15506488269543164</x:v>
+      </x:c>
+      <x:c r="G12" s="13" t="n">
+        <x:v>0.0081765583185379</x:v>
+      </x:c>
+      <x:c r="H12" s="12" t="n">
+        <x:v>-0.3128163233905591</x:v>
+      </x:c>
+      <x:c r="I12" s="11" t="n">
+        <x:v>-0.3212700209602253</x:v>
+      </x:c>
+      <x:c r="J12" s="11" t="n">
+        <x:v>1.427256445191111</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="23" customHeight="1">
+      <x:c r="A13" s="2" t="str">
+        <x:v>THINK + mixer / Daily / new five seeds</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D13" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="n">
+        <x:v>0.4853858869659288</x:v>
+      </x:c>
+      <x:c r="F13" s="12" t="n">
+        <x:v>0.1379016744844486</x:v>
+      </x:c>
+      <x:c r="G13" s="13" t="n">
+        <x:v>0.0081765583185379</x:v>
+      </x:c>
+      <x:c r="H13" s="12" t="n">
+        <x:v>-0.3216483863456999</x:v>
+      </x:c>
+      <x:c r="I13" s="11" t="n">
+        <x:v>-0.3707526236517362</x:v>
+      </x:c>
+      <x:c r="J13" s="11" t="n">
+        <x:v>1.3721975317245534</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="23" customHeight="1">
+      <x:c r="A14" s="2" t="str">
+        <x:v>THINK + mixer / Daily / new five seeds</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D14" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="n">
+        <x:v>0.38361093775345634</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="n">
+        <x:v>0.10440763397853314</x:v>
+      </x:c>
+      <x:c r="G14" s="13" t="n">
+        <x:v>0.0081765583185379</x:v>
+      </x:c>
+      <x:c r="H14" s="12" t="n">
+        <x:v>-0.3389741831879073</x:v>
+      </x:c>
+      <x:c r="I14" s="11" t="n">
+        <x:v>-0.4697942037353103</x:v>
+      </x:c>
+      <x:c r="J14" s="11" t="n">
+        <x:v>1.2649342733662945</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="23" customHeight="1">
+      <x:c r="A15" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 7</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D15" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="n">
+        <x:v>0.451772352519994</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="n">
+        <x:v>0.12771908055830827</x:v>
+      </x:c>
+      <x:c r="G15" s="13" t="n">
+        <x:v>0.0056579793579048</x:v>
+      </x:c>
+      <x:c r="H15" s="12" t="n">
+        <x:v>-0.36589086764733814</x:v>
+      </x:c>
+      <x:c r="I15" s="11" t="n">
+        <x:v>-0.371086060798281</x:v>
+      </x:c>
+      <x:c r="J15" s="11" t="n">
+        <x:v>1.3240632793134897</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="23" customHeight="1">
+      <x:c r="A16" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 19</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D16" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="11" t="n">
+        <x:v>0.675515548035325</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="n">
+        <x:v>0.2117838580308752</x:v>
+      </x:c>
+      <x:c r="G16" s="13" t="n">
+        <x:v>0.0159965075987652</x:v>
+      </x:c>
+      <x:c r="H16" s="12" t="n">
+        <x:v>-0.35016580545575415</x:v>
+      </x:c>
+      <x:c r="I16" s="11" t="n">
+        <x:v>-0.181948720482144</x:v>
+      </x:c>
+      <x:c r="J16" s="11" t="n">
+        <x:v>1.5866607142284386</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="23" customHeight="1">
+      <x:c r="A17" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 42</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D17" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="n">
+        <x:v>0.3752257016228017</x:v>
+      </x:c>
+      <x:c r="F17" s="12" t="n">
+        <x:v>0.10238017595693766</x:v>
+      </x:c>
+      <x:c r="G17" s="13" t="n">
+        <x:v>0.0010043238069504</x:v>
+      </x:c>
+      <x:c r="H17" s="12" t="n">
+        <x:v>-0.35526812537531194</x:v>
+      </x:c>
+      <x:c r="I17" s="11" t="n">
+        <x:v>-0.4172460956457126</x:v>
+      </x:c>
+      <x:c r="J17" s="11" t="n">
+        <x:v>1.213139670241272</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="23" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 61</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="D18" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="11" t="n">
+        <x:v>0.32879060283636136</x:v>
+      </x:c>
+      <x:c r="F18" s="12" t="n">
+        <x:v>0.08487372637296517</x:v>
+      </x:c>
+      <x:c r="G18" s="13" t="n">
+        <x:v>0.0011625152415479</x:v>
+      </x:c>
+      <x:c r="H18" s="12" t="n">
+        <x:v>-0.2992582621964539</x:v>
+      </x:c>
+      <x:c r="I18" s="11" t="n">
+        <x:v>-0.4949084383520276</x:v>
+      </x:c>
+      <x:c r="J18" s="11" t="n">
+        <x:v>1.197683018889803</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="23" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 97</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="D19" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="11" t="n">
+        <x:v>0.42997242045042317</x:v>
+      </x:c>
+      <x:c r="F19" s="12" t="n">
+        <x:v>0.12437819302527889</x:v>
+      </x:c>
+      <x:c r="G19" s="13" t="n">
+        <x:v>0.0104141466654526</x:v>
+      </x:c>
+      <x:c r="H19" s="12" t="n">
+        <x:v>-0.36998232779608464</x:v>
+      </x:c>
+      <x:c r="I19" s="11" t="n">
+        <x:v>-0.3806352033187475</x:v>
+      </x:c>
+      <x:c r="J19" s="11" t="n">
+        <x:v>1.2896919535622589</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="23" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 1828801906</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>1828801906</x:v>
+      </x:c>
+      <x:c r="D20" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E20" s="11" t="n">
+        <x:v>0.2816924388203836</x:v>
+      </x:c>
+      <x:c r="F20" s="12" t="n">
+        <x:v>0.07174941575180441</x:v>
+      </x:c>
+      <x:c r="G20" s="13" t="n">
+        <x:v>0.0061811440437555</x:v>
+      </x:c>
+      <x:c r="H20" s="12" t="n">
+        <x:v>-0.3511543801336503</x:v>
+      </x:c>
+      <x:c r="I20" s="11" t="n">
+        <x:v>-0.5574617190774849</x:v>
+      </x:c>
+      <x:c r="J20" s="11" t="n">
+        <x:v>1.157038480804428</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="23" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 1868046758</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>1868046758</x:v>
+      </x:c>
+      <x:c r="D21" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E21" s="11" t="n">
+        <x:v>0.35007485876182</x:v>
+      </x:c>
+      <x:c r="F21" s="12" t="n">
+        <x:v>0.09376325874672692</x:v>
+      </x:c>
+      <x:c r="G21" s="13" t="n">
+        <x:v>0.0079484536902092</x:v>
+      </x:c>
+      <x:c r="H21" s="12" t="n">
+        <x:v>-0.3313114076599566</x:v>
+      </x:c>
+      <x:c r="I21" s="11" t="n">
+        <x:v>-0.5199253149961828</x:v>
+      </x:c>
+      <x:c r="J21" s="11" t="n">
+        <x:v>1.2591090081955676</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="23" customHeight="1">
+      <x:c r="A22" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 239154507</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>239154507</x:v>
+      </x:c>
+      <x:c r="D22" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E22" s="11" t="n">
+        <x:v>0.2924415858718266</x:v>
+      </x:c>
+      <x:c r="F22" s="12" t="n">
+        <x:v>0.07517398416738838</x:v>
+      </x:c>
+      <x:c r="G22" s="13" t="n">
+        <x:v>0.0180308527469106</x:v>
+      </x:c>
+      <x:c r="H22" s="12" t="n">
+        <x:v>-0.312665146112988</x:v>
+      </x:c>
+      <x:c r="I22" s="11" t="n">
+        <x:v>-0.5507325542081437</x:v>
+      </x:c>
+      <x:c r="J22" s="11" t="n">
+        <x:v>1.172854863533532</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="23" customHeight="1">
+      <x:c r="A23" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 287727767</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>287727767</x:v>
+      </x:c>
+      <x:c r="D23" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E23" s="11" t="n">
+        <x:v>0.23485817962147837</x:v>
+      </x:c>
+      <x:c r="F23" s="12" t="n">
+        <x:v>0.057597650875556045</x:v>
+      </x:c>
+      <x:c r="G23" s="13" t="n">
+        <x:v>-0.0075379670902185</x:v>
+      </x:c>
+      <x:c r="H23" s="12" t="n">
+        <x:v>-0.34468717132654303</x:v>
+      </x:c>
+      <x:c r="I23" s="11" t="n">
+        <x:v>-0.5843193209042872</x:v>
+      </x:c>
+      <x:c r="J23" s="11" t="n">
+        <x:v>1.105033702517185</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="23" customHeight="1">
+      <x:c r="A24" s="2" t="str">
+        <x:v>THINK + mixer / Daily / seed 981756941</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
+        <x:v>981756941</x:v>
+      </x:c>
+      <x:c r="D24" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E24" s="11" t="n">
+        <x:v>0.33307987512987874</x:v>
+      </x:c>
+      <x:c r="F24" s="12" t="n">
+        <x:v>0.0880857657769998</x:v>
+      </x:c>
+      <x:c r="G24" s="13" t="n">
+        <x:v>0.0090966434113513</x:v>
+      </x:c>
+      <x:c r="H24" s="12" t="n">
+        <x:v>-0.38823021237886457</x:v>
+      </x:c>
+      <x:c r="I24" s="11" t="n">
+        <x:v>-0.5305374161218038</x:v>
+      </x:c>
+      <x:c r="J24" s="11" t="n">
+        <x:v>1.2200120261337728</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="23" customHeight="1">
+      <x:c r="A25" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / ten seeds</x:v>
+      </x:c>
+      <x:c r="B25" s="2" t="str">
+        <x:v>Primary ten-seed ensemble</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D25" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="n">
+        <x:v>0.4882238564367686</x:v>
+      </x:c>
+      <x:c r="F25" s="12" t="n">
+        <x:v>0.14226921456410785</x:v>
+      </x:c>
+      <x:c r="G25" s="13" t="n">
+        <x:v>0.0035727536866006</x:v>
+      </x:c>
+      <x:c r="H25" s="12" t="n">
+        <x:v>-0.4011704221619038</x:v>
+      </x:c>
+      <x:c r="I25" s="11" t="n">
+        <x:v>-0.3665240836934171</x:v>
+      </x:c>
+      <x:c r="J25" s="11" t="n">
+        <x:v>1.3827586125394058</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="23" customHeight="1">
+      <x:c r="A26" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / ten seeds</x:v>
+      </x:c>
+      <x:c r="B26" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D26" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="n">
+        <x:v>0.44152679493849595</x:v>
+      </x:c>
+      <x:c r="F26" s="12" t="n">
+        <x:v>0.12585436770153957</x:v>
+      </x:c>
+      <x:c r="G26" s="13" t="n">
+        <x:v>0.0035727536866006</x:v>
+      </x:c>
+      <x:c r="H26" s="12" t="n">
+        <x:v>-0.4095001866472444</x:v>
+      </x:c>
+      <x:c r="I26" s="11" t="n">
+        <x:v>-0.4122543827449981</x:v>
+      </x:c>
+      <x:c r="J26" s="11" t="n">
+        <x:v>1.333197650450252</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="23" customHeight="1">
+      <x:c r="A27" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / ten seeds</x:v>
+      </x:c>
+      <x:c r="B27" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D27" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E27" s="11" t="n">
+        <x:v>0.34840574042158157</x:v>
+      </x:c>
+      <x:c r="F27" s="12" t="n">
+        <x:v>0.09379335903442805</x:v>
+      </x:c>
+      <x:c r="G27" s="13" t="n">
+        <x:v>0.0035727536866006</x:v>
+      </x:c>
+      <x:c r="H27" s="12" t="n">
+        <x:v>-0.4257939670520411</x:v>
+      </x:c>
+      <x:c r="I27" s="11" t="n">
+        <x:v>-0.5004807569725006</x:v>
+      </x:c>
+      <x:c r="J27" s="11" t="n">
+        <x:v>1.2390482698013832</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="23" customHeight="1">
+      <x:c r="A28" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / original five seeds</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="str">
+        <x:v>Seed-subgroup diagnostic</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D28" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E28" s="11" t="n">
+        <x:v>0.6024624994600978</x:v>
+      </x:c>
+      <x:c r="F28" s="12" t="n">
+        <x:v>0.1860236058844805</x:v>
+      </x:c>
+      <x:c r="G28" s="13" t="n">
+        <x:v>0.0063408707312977</x:v>
+      </x:c>
+      <x:c r="H28" s="12" t="n">
+        <x:v>-0.37161827435781014</x:v>
+      </x:c>
+      <x:c r="I28" s="11" t="n">
+        <x:v>-0.2193536466130756</x:v>
+      </x:c>
+      <x:c r="J28" s="11" t="n">
+        <x:v>1.4754691689101456</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="23" customHeight="1">
+      <x:c r="A29" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / original five seeds</x:v>
+      </x:c>
+      <x:c r="B29" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D29" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E29" s="11" t="n">
+        <x:v>0.5439003694396268</x:v>
+      </x:c>
+      <x:c r="F29" s="12" t="n">
+        <x:v>0.16423962439349374</x:v>
+      </x:c>
+      <x:c r="G29" s="13" t="n">
+        <x:v>0.0063408707312977</x:v>
+      </x:c>
+      <x:c r="H29" s="12" t="n">
+        <x:v>-0.37883413100760377</x:v>
+      </x:c>
+      <x:c r="I29" s="11" t="n">
+        <x:v>-0.2787750466638217</x:v>
+      </x:c>
+      <x:c r="J29" s="11" t="n">
+        <x:v>1.4151502922965036</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="23" customHeight="1">
+      <x:c r="A30" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / original five seeds</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D30" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E30" s="11" t="n">
+        <x:v>0.42746093351235087</x:v>
+      </x:c>
+      <x:c r="F30" s="12" t="n">
+        <x:v>0.12202175377108052</x:v>
+      </x:c>
+      <x:c r="G30" s="13" t="n">
+        <x:v>0.0063408707312977</x:v>
+      </x:c>
+      <x:c r="H30" s="12" t="n">
+        <x:v>-0.39927809458058583</x:v>
+      </x:c>
+      <x:c r="I30" s="11" t="n">
+        <x:v>-0.396305524709984</x:v>
+      </x:c>
+      <x:c r="J30" s="11" t="n">
+        <x:v>1.2932787313501206</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="23" customHeight="1">
+      <x:c r="A31" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / new five seeds</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>Seed-subgroup diagnostic</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D31" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E31" s="11" t="n">
+        <x:v>0.47398709120623245</x:v>
+      </x:c>
+      <x:c r="F31" s="12" t="n">
+        <x:v>0.13432742993395266</x:v>
+      </x:c>
+      <x:c r="G31" s="13" t="n">
+        <x:v>0.0060933322472734</x:v>
+      </x:c>
+      <x:c r="H31" s="12" t="n">
+        <x:v>-0.33121069853341756</x:v>
+      </x:c>
+      <x:c r="I31" s="11" t="n">
+        <x:v>-0.386761700440253</x:v>
+      </x:c>
+      <x:c r="J31" s="11" t="n">
+        <x:v>1.381458473720616</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="23" customHeight="1">
+      <x:c r="A32" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / new five seeds</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D32" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E32" s="11" t="n">
+        <x:v>0.4241382580397084</x:v>
+      </x:c>
+      <x:c r="F32" s="12" t="n">
+        <x:v>0.11778463164377986</x:v>
+      </x:c>
+      <x:c r="G32" s="13" t="n">
+        <x:v>0.0060933322472734</x:v>
+      </x:c>
+      <x:c r="H32" s="12" t="n">
+        <x:v>-0.3408805238495276</x:v>
+      </x:c>
+      <x:c r="I32" s="11" t="n">
+        <x:v>-0.4377592137528165</x:v>
+      </x:c>
+      <x:c r="J32" s="11" t="n">
+        <x:v>1.329135060854373</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="23" customHeight="1">
+      <x:c r="A33" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / new five seeds</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D33" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E33" s="11" t="n">
+        <x:v>0.3249594876047447</x:v>
+      </x:c>
+      <x:c r="F33" s="12" t="n">
+        <x:v>0.08554081848356143</x:v>
+      </x:c>
+      <x:c r="G33" s="13" t="n">
+        <x:v>0.0060933322472734</x:v>
+      </x:c>
+      <x:c r="H33" s="12" t="n">
+        <x:v>-0.35975837843960246</x:v>
+      </x:c>
+      <x:c r="I33" s="11" t="n">
+        <x:v>-0.5383162643005797</x:v>
+      </x:c>
+      <x:c r="J33" s="11" t="n">
+        <x:v>1.223652126907471</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="23" customHeight="1">
+      <x:c r="A34" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 7</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D34" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E34" s="11" t="n">
+        <x:v>0.48501170336444965</x:v>
+      </x:c>
+      <x:c r="F34" s="12" t="n">
+        <x:v>0.13925167920324744</x:v>
+      </x:c>
+      <x:c r="G34" s="13" t="n">
+        <x:v>0.0059837199190701</x:v>
+      </x:c>
+      <x:c r="H34" s="12" t="n">
+        <x:v>-0.36638456690018817</x:v>
+      </x:c>
+      <x:c r="I34" s="11" t="n">
+        <x:v>-0.3464886186683982</x:v>
+      </x:c>
+      <x:c r="J34" s="11" t="n">
+        <x:v>1.3794055744753233</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="23" customHeight="1">
+      <x:c r="A35" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 19</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D35" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="11" t="n">
+        <x:v>0.6652452743812108</x:v>
+      </x:c>
+      <x:c r="F35" s="12" t="n">
+        <x:v>0.20842431858360033</x:v>
+      </x:c>
+      <x:c r="G35" s="13" t="n">
+        <x:v>0.0155257475798709</x:v>
+      </x:c>
+      <x:c r="H35" s="12" t="n">
+        <x:v>-0.34970741525036464</x:v>
+      </x:c>
+      <x:c r="I35" s="11" t="n">
+        <x:v>-0.1785192983564605</x:v>
+      </x:c>
+      <x:c r="J35" s="11" t="n">
+        <x:v>1.5646147408214075</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="23" customHeight="1">
+      <x:c r="A36" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 42</x:v>
+      </x:c>
+      <x:c r="B36" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D36" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E36" s="11" t="n">
+        <x:v>0.21087489424286637</x:v>
+      </x:c>
+      <x:c r="F36" s="12" t="n">
+        <x:v>0.04841710377679416</x:v>
+      </x:c>
+      <x:c r="G36" s="13" t="n">
+        <x:v>-0.0004745281933009</x:v>
+      </x:c>
+      <x:c r="H36" s="12" t="n">
+        <x:v>-0.41296862196140793</x:v>
+      </x:c>
+      <x:c r="I36" s="11" t="n">
+        <x:v>-0.5959249877321467</x:v>
+      </x:c>
+      <x:c r="J36" s="11" t="n">
+        <x:v>1.0650913476907198</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="23" customHeight="1">
+      <x:c r="A37" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 61</x:v>
+      </x:c>
+      <x:c r="B37" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="D37" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E37" s="11" t="n">
+        <x:v>0.30524225792589266</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="n">
+        <x:v>0.07823713762827228</x:v>
+      </x:c>
+      <x:c r="G37" s="13" t="n">
+        <x:v>0.0001391371640105</x:v>
+      </x:c>
+      <x:c r="H37" s="12" t="n">
+        <x:v>-0.29486120779323033</x:v>
+      </x:c>
+      <x:c r="I37" s="11" t="n">
+        <x:v>-0.5135948820036568</x:v>
+      </x:c>
+      <x:c r="J37" s="11" t="n">
+        <x:v>1.160728162649754</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="23" customHeight="1">
+      <x:c r="A38" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 97</x:v>
+      </x:c>
+      <x:c r="B38" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C38" s="2" t="str">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="D38" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E38" s="11" t="n">
+        <x:v>0.5270981523418959</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="n">
+        <x:v>0.16118254079930536</x:v>
+      </x:c>
+      <x:c r="G38" s="13" t="n">
+        <x:v>0.0104919878464046</x:v>
+      </x:c>
+      <x:c r="H38" s="12" t="n">
+        <x:v>-0.36643276887467824</x:v>
+      </x:c>
+      <x:c r="I38" s="11" t="n">
+        <x:v>-0.2915395703249874</x:v>
+      </x:c>
+      <x:c r="J38" s="11" t="n">
+        <x:v>1.388438935328502</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="23" customHeight="1">
+      <x:c r="A39" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 1828801906</x:v>
+      </x:c>
+      <x:c r="B39" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C39" s="2" t="str">
+        <x:v>1828801906</x:v>
+      </x:c>
+      <x:c r="D39" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E39" s="11" t="n">
+        <x:v>0.3321322708832354</x:v>
+      </x:c>
+      <x:c r="F39" s="12" t="n">
+        <x:v>0.08760003388696512</x:v>
+      </x:c>
+      <x:c r="G39" s="13" t="n">
+        <x:v>0.0055655510688376</x:v>
+      </x:c>
+      <x:c r="H39" s="12" t="n">
+        <x:v>-0.337424551049915</x:v>
+      </x:c>
+      <x:c r="I39" s="11" t="n">
+        <x:v>-0.5032468153811421</x:v>
+      </x:c>
+      <x:c r="J39" s="11" t="n">
+        <x:v>1.2002298875062265</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="23" customHeight="1">
+      <x:c r="A40" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 1868046758</x:v>
+      </x:c>
+      <x:c r="B40" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C40" s="2" t="str">
+        <x:v>1868046758</x:v>
+      </x:c>
+      <x:c r="D40" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E40" s="11" t="n">
+        <x:v>0.32461886923457667</x:v>
+      </x:c>
+      <x:c r="F40" s="12" t="n">
+        <x:v>0.0855648757870327</x:v>
+      </x:c>
+      <x:c r="G40" s="13" t="n">
+        <x:v>0.0067480848720222</x:v>
+      </x:c>
+      <x:c r="H40" s="12" t="n">
+        <x:v>-0.3337372453387013</x:v>
+      </x:c>
+      <x:c r="I40" s="11" t="n">
+        <x:v>-0.5479067845378339</x:v>
+      </x:c>
+      <x:c r="J40" s="11" t="n">
+        <x:v>1.2332654915903902</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="23" customHeight="1">
+      <x:c r="A41" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 239154507</x:v>
+      </x:c>
+      <x:c r="B41" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C41" s="2" t="str">
+        <x:v>239154507</x:v>
+      </x:c>
+      <x:c r="D41" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E41" s="11" t="n">
+        <x:v>0.26111023242279907</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="n">
+        <x:v>0.06509118546049615</x:v>
+      </x:c>
+      <x:c r="G41" s="13" t="n">
+        <x:v>0.0170785099152719</x:v>
+      </x:c>
+      <x:c r="H41" s="12" t="n">
+        <x:v>-0.3505969565818564</x:v>
+      </x:c>
+      <x:c r="I41" s="11" t="n">
+        <x:v>-0.5662656472947968</x:v>
+      </x:c>
+      <x:c r="J41" s="11" t="n">
+        <x:v>1.129561641486491</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="23" customHeight="1">
+      <x:c r="A42" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 287727767</x:v>
+      </x:c>
+      <x:c r="B42" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C42" s="2" t="str">
+        <x:v>287727767</x:v>
+      </x:c>
+      <x:c r="D42" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E42" s="11" t="n">
+        <x:v>0.05037800688007422</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="n">
+        <x:v>0.005359826819045703</x:v>
+      </x:c>
+      <x:c r="G42" s="13" t="n">
+        <x:v>-0.0095132247444563</x:v>
+      </x:c>
+      <x:c r="H42" s="12" t="n">
+        <x:v>-0.35909026839567526</x:v>
+      </x:c>
+      <x:c r="I42" s="11" t="n">
+        <x:v>-0.7709234060038243</x:v>
+      </x:c>
+      <x:c r="J42" s="11" t="n">
+        <x:v>0.8949094474195635</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="23" customHeight="1">
+      <x:c r="A43" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH / seed 981756941</x:v>
+      </x:c>
+      <x:c r="B43" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C43" s="2" t="str">
+        <x:v>981756941</x:v>
+      </x:c>
+      <x:c r="D43" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E43" s="11" t="n">
+        <x:v>0.3230542855118197</x:v>
+      </x:c>
+      <x:c r="F43" s="12" t="n">
+        <x:v>0.08472417275862992</x:v>
+      </x:c>
+      <x:c r="G43" s="13" t="n">
+        <x:v>0.0062356349114222</x:v>
+      </x:c>
+      <x:c r="H43" s="12" t="n">
+        <x:v>-0.37402830275000043</x:v>
+      </x:c>
+      <x:c r="I43" s="11" t="n">
+        <x:v>-0.5350377187352707</x:v>
+      </x:c>
+      <x:c r="J43" s="11" t="n">
+        <x:v>1.200804563032812</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="23" customHeight="1">
+      <x:c r="A44" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / ten seeds</x:v>
+      </x:c>
+      <x:c r="B44" s="2" t="str">
+        <x:v>Primary ten-seed ensemble</x:v>
+      </x:c>
+      <x:c r="C44" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D44" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E44" s="11" t="n">
+        <x:v>0.5191500032056338</x:v>
+      </x:c>
+      <x:c r="F44" s="12" t="n">
+        <x:v>0.15356400976834336</x:v>
+      </x:c>
+      <x:c r="G44" s="13" t="n">
+        <x:v>0.0037740295593641</x:v>
+      </x:c>
+      <x:c r="H44" s="12" t="n">
+        <x:v>-0.3832320310700549</x:v>
+      </x:c>
+      <x:c r="I44" s="11" t="n">
+        <x:v>-0.3452746799425182</x:v>
+      </x:c>
+      <x:c r="J44" s="11" t="n">
+        <x:v>1.425365964092924</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="23" customHeight="1">
+      <x:c r="A45" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / ten seeds</x:v>
+      </x:c>
+      <x:c r="B45" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C45" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D45" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E45" s="11" t="n">
+        <x:v>0.47421383764089986</x:v>
+      </x:c>
+      <x:c r="F45" s="12" t="n">
+        <x:v>0.13755628053798521</x:v>
+      </x:c>
+      <x:c r="G45" s="13" t="n">
+        <x:v>0.0037740295593641</x:v>
+      </x:c>
+      <x:c r="H45" s="12" t="n">
+        <x:v>-0.39181158706472907</x:v>
+      </x:c>
+      <x:c r="I45" s="11" t="n">
+        <x:v>-0.3904587438227595</x:v>
+      </x:c>
+      <x:c r="J45" s="11" t="n">
+        <x:v>1.3788166270906903</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="23" customHeight="1">
+      <x:c r="A46" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / ten seeds</x:v>
+      </x:c>
+      <x:c r="B46" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C46" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D46" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E46" s="11" t="n">
+        <x:v>0.3847081377885628</x:v>
+      </x:c>
+      <x:c r="F46" s="12" t="n">
+        <x:v>0.10629628098271345</x:v>
+      </x:c>
+      <x:c r="G46" s="13" t="n">
+        <x:v>0.0037740295593641</x:v>
+      </x:c>
+      <x:c r="H46" s="12" t="n">
+        <x:v>-0.40855548586069523</x:v>
+      </x:c>
+      <x:c r="I46" s="11" t="n">
+        <x:v>-0.4765735124669309</x:v>
+      </x:c>
+      <x:c r="J46" s="11" t="n">
+        <x:v>1.2866983644622814</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="23" customHeight="1">
+      <x:c r="A47" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / original five seeds</x:v>
+      </x:c>
+      <x:c r="B47" s="2" t="str">
+        <x:v>Seed-subgroup diagnostic</x:v>
+      </x:c>
+      <x:c r="C47" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D47" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E47" s="11" t="n">
+        <x:v>0.7002722836906295</x:v>
+      </x:c>
+      <x:c r="F47" s="12" t="n">
+        <x:v>0.22385598411825272</x:v>
+      </x:c>
+      <x:c r="G47" s="13" t="n">
+        <x:v>0.0060550276299253</x:v>
+      </x:c>
+      <x:c r="H47" s="12" t="n">
+        <x:v>-0.35013286984215053</x:v>
+      </x:c>
+      <x:c r="I47" s="11" t="n">
+        <x:v>-0.1393513711221214</x:v>
+      </x:c>
+      <x:c r="J47" s="11" t="n">
+        <x:v>1.5935183268359752</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="23" customHeight="1">
+      <x:c r="A48" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / original five seeds</x:v>
+      </x:c>
+      <x:c r="B48" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C48" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D48" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E48" s="11" t="n">
+        <x:v>0.6444365016021609</x:v>
+      </x:c>
+      <x:c r="F48" s="12" t="n">
+        <x:v>0.20239039285137214</x:v>
+      </x:c>
+      <x:c r="G48" s="13" t="n">
+        <x:v>0.0060550276299253</x:v>
+      </x:c>
+      <x:c r="H48" s="12" t="n">
+        <x:v>-0.36173396978854433</x:v>
+      </x:c>
+      <x:c r="I48" s="11" t="n">
+        <x:v>-0.1948047074662189</x:v>
+      </x:c>
+      <x:c r="J48" s="11" t="n">
+        <x:v>1.5368796185682068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="23" customHeight="1">
+      <x:c r="A49" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / original five seeds</x:v>
+      </x:c>
+      <x:c r="B49" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C49" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D49" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E49" s="11" t="n">
+        <x:v>0.5334433077953485</x:v>
+      </x:c>
+      <x:c r="F49" s="12" t="n">
+        <x:v>0.16074625312457422</x:v>
+      </x:c>
+      <x:c r="G49" s="13" t="n">
+        <x:v>0.0060550276299253</x:v>
+      </x:c>
+      <x:c r="H49" s="12" t="n">
+        <x:v>-0.3841816276079658</x:v>
+      </x:c>
+      <x:c r="I49" s="11" t="n">
+        <x:v>-0.2990173518394353</x:v>
+      </x:c>
+      <x:c r="J49" s="11" t="n">
+        <x:v>1.4172815385834074</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="23" customHeight="1">
+      <x:c r="A50" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / new five seeds</x:v>
+      </x:c>
+      <x:c r="B50" s="2" t="str">
+        <x:v>Seed-subgroup diagnostic</x:v>
+      </x:c>
+      <x:c r="C50" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D50" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E50" s="11" t="n">
+        <x:v>0.4802168579045056</x:v>
+      </x:c>
+      <x:c r="F50" s="12" t="n">
+        <x:v>0.13693671292731538</x:v>
+      </x:c>
+      <x:c r="G50" s="13" t="n">
+        <x:v>0.0067411410003181</x:v>
+      </x:c>
+      <x:c r="H50" s="12" t="n">
+        <x:v>-0.34402710440142015</x:v>
+      </x:c>
+      <x:c r="I50" s="11" t="n">
+        <x:v>-0.3816345022820374</x:v>
+      </x:c>
+      <x:c r="J50" s="11" t="n">
+        <x:v>1.3651643080407354</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="23" customHeight="1">
+      <x:c r="A51" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / new five seeds</x:v>
+      </x:c>
+      <x:c r="B51" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C51" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D51" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E51" s="11" t="n">
+        <x:v>0.43174834999214934</x:v>
+      </x:c>
+      <x:c r="F51" s="12" t="n">
+        <x:v>0.12067424251752772</x:v>
+      </x:c>
+      <x:c r="G51" s="13" t="n">
+        <x:v>0.0067411410003181</x:v>
+      </x:c>
+      <x:c r="H51" s="12" t="n">
+        <x:v>-0.35026788229939765</x:v>
+      </x:c>
+      <x:c r="I51" s="11" t="n">
+        <x:v>-0.4267797848169209</x:v>
+      </x:c>
+      <x:c r="J51" s="11" t="n">
+        <x:v>1.3174016224121232</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="23" customHeight="1">
+      <x:c r="A52" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / new five seeds</x:v>
+      </x:c>
+      <x:c r="B52" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C52" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D52" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E52" s="11" t="n">
+        <x:v>0.33521906696957643</x:v>
+      </x:c>
+      <x:c r="F52" s="12" t="n">
+        <x:v>0.08893907776561483</x:v>
+      </x:c>
+      <x:c r="G52" s="13" t="n">
+        <x:v>0.0067411410003181</x:v>
+      </x:c>
+      <x:c r="H52" s="12" t="n">
+        <x:v>-0.3625471235713813</x:v>
+      </x:c>
+      <x:c r="I52" s="11" t="n">
+        <x:v>-0.5161496684257989</x:v>
+      </x:c>
+      <x:c r="J52" s="11" t="n">
+        <x:v>1.2188872881530386</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="23" customHeight="1">
+      <x:c r="A53" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 7</x:v>
+      </x:c>
+      <x:c r="B53" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C53" s="2" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D53" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E53" s="11" t="n">
+        <x:v>0.5651208064997345</x:v>
+      </x:c>
+      <x:c r="F53" s="12" t="n">
+        <x:v>0.1672729424762129</x:v>
+      </x:c>
+      <x:c r="G53" s="13" t="n">
+        <x:v>0.0063615355315577</x:v>
+      </x:c>
+      <x:c r="H53" s="12" t="n">
+        <x:v>-0.345262441493253</x:v>
+      </x:c>
+      <x:c r="I53" s="11" t="n">
+        <x:v>-0.268171961847896</x:v>
+      </x:c>
+      <x:c r="J53" s="11" t="n">
+        <x:v>1.4675458483975024</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="23" customHeight="1">
+      <x:c r="A54" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 19</x:v>
+      </x:c>
+      <x:c r="B54" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C54" s="2" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D54" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E54" s="11" t="n">
+        <x:v>0.6633996784687809</x:v>
+      </x:c>
+      <x:c r="F54" s="12" t="n">
+        <x:v>0.20829665477210685</x:v>
+      </x:c>
+      <x:c r="G54" s="13" t="n">
+        <x:v>0.0164529890541201</x:v>
+      </x:c>
+      <x:c r="H54" s="12" t="n">
+        <x:v>-0.33730260262881373</x:v>
+      </x:c>
+      <x:c r="I54" s="11" t="n">
+        <x:v>-0.193368025612255</x:v>
+      </x:c>
+      <x:c r="J54" s="11" t="n">
+        <x:v>1.5564720014313354</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="23" customHeight="1">
+      <x:c r="A55" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 42</x:v>
+      </x:c>
+      <x:c r="B55" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C55" s="2" t="str">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D55" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E55" s="11" t="n">
+        <x:v>0.39237718558282303</x:v>
+      </x:c>
+      <x:c r="F55" s="12" t="n">
+        <x:v>0.1084504498806517</x:v>
+      </x:c>
+      <x:c r="G55" s="13" t="n">
+        <x:v>-0.0006562646522129</x:v>
+      </x:c>
+      <x:c r="H55" s="12" t="n">
+        <x:v>-0.3753998166104128</x:v>
+      </x:c>
+      <x:c r="I55" s="11" t="n">
+        <x:v>-0.4558393002608228</x:v>
+      </x:c>
+      <x:c r="J55" s="11" t="n">
+        <x:v>1.2681569290944958</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="23" customHeight="1">
+      <x:c r="A56" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 61</x:v>
+      </x:c>
+      <x:c r="B56" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C56" s="2" t="str">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="D56" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E56" s="11" t="n">
+        <x:v>0.25589018244834577</x:v>
+      </x:c>
+      <x:c r="F56" s="12" t="n">
+        <x:v>0.06440634161885768</x:v>
+      </x:c>
+      <x:c r="G56" s="13" t="n">
+        <x:v>0.0004113084865772</x:v>
+      </x:c>
+      <x:c r="H56" s="12" t="n">
+        <x:v>-0.3218415618282522</x:v>
+      </x:c>
+      <x:c r="I56" s="11" t="n">
+        <x:v>-0.5575047850221089</x:v>
+      </x:c>
+      <x:c r="J56" s="11" t="n">
+        <x:v>1.108965480122264</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="23" customHeight="1">
+      <x:c r="A57" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 97</x:v>
+      </x:c>
+      <x:c r="B57" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C57" s="2" t="str">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="D57" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E57" s="11" t="n">
+        <x:v>0.5476847126772674</x:v>
+      </x:c>
+      <x:c r="F57" s="12" t="n">
+        <x:v>0.1704475243928276</x:v>
+      </x:c>
+      <x:c r="G57" s="13" t="n">
+        <x:v>0.0105792873853562</x:v>
+      </x:c>
+      <x:c r="H57" s="12" t="n">
+        <x:v>-0.35018193590020075</x:v>
+      </x:c>
+      <x:c r="I57" s="11" t="n">
+        <x:v>-0.2636992104606427</x:v>
+      </x:c>
+      <x:c r="J57" s="11" t="n">
+        <x:v>1.3956411834916589</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="23" customHeight="1">
+      <x:c r="A58" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 1828801906</x:v>
+      </x:c>
+      <x:c r="B58" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C58" s="2" t="str">
+        <x:v>1828801906</x:v>
+      </x:c>
+      <x:c r="D58" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E58" s="11" t="n">
+        <x:v>0.32187579185126447</x:v>
+      </x:c>
+      <x:c r="F58" s="12" t="n">
+        <x:v>0.08437105849495813</x:v>
+      </x:c>
+      <x:c r="G58" s="13" t="n">
+        <x:v>0.0055545738930387</x:v>
+      </x:c>
+      <x:c r="H58" s="12" t="n">
+        <x:v>-0.3404805734197617</x:v>
+      </x:c>
+      <x:c r="I58" s="11" t="n">
+        <x:v>-0.5137563660002348</x:v>
+      </x:c>
+      <x:c r="J58" s="11" t="n">
+        <x:v>1.1862888589223275</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="23" customHeight="1">
+      <x:c r="A59" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 1868046758</x:v>
+      </x:c>
+      <x:c r="B59" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C59" s="2" t="str">
+        <x:v>1868046758</x:v>
+      </x:c>
+      <x:c r="D59" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E59" s="11" t="n">
+        <x:v>0.3652305265727224</x:v>
+      </x:c>
+      <x:c r="F59" s="12" t="n">
+        <x:v>0.0989923930861166</x:v>
+      </x:c>
+      <x:c r="G59" s="13" t="n">
+        <x:v>0.0052742101932949</x:v>
+      </x:c>
+      <x:c r="H59" s="12" t="n">
+        <x:v>-0.34549500762090524</x:v>
+      </x:c>
+      <x:c r="I59" s="11" t="n">
+        <x:v>-0.509261358068551</x:v>
+      </x:c>
+      <x:c r="J59" s="11" t="n">
+        <x:v>1.2713388035376054</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="23" customHeight="1">
+      <x:c r="A60" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 239154507</x:v>
+      </x:c>
+      <x:c r="B60" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C60" s="2" t="str">
+        <x:v>239154507</x:v>
+      </x:c>
+      <x:c r="D60" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E60" s="11" t="n">
+        <x:v>0.24474757972220723</x:v>
+      </x:c>
+      <x:c r="F60" s="12" t="n">
+        <x:v>0.05988797781135674</x:v>
+      </x:c>
+      <x:c r="G60" s="13" t="n">
+        <x:v>0.0183932188439569</x:v>
+      </x:c>
+      <x:c r="H60" s="12" t="n">
+        <x:v>-0.35299989362954565</x:v>
+      </x:c>
+      <x:c r="I60" s="11" t="n">
+        <x:v>-0.5769881567681804</x:v>
+      </x:c>
+      <x:c r="J60" s="11" t="n">
+        <x:v>1.099505711855033</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="23" customHeight="1">
+      <x:c r="A61" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 287727767</x:v>
+      </x:c>
+      <x:c r="B61" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C61" s="2" t="str">
+        <x:v>287727767</x:v>
+      </x:c>
+      <x:c r="D61" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E61" s="11" t="n">
+        <x:v>0.16519122435153094</x:v>
+      </x:c>
+      <x:c r="F61" s="12" t="n">
+        <x:v>0.03760996855692404</x:v>
+      </x:c>
+      <x:c r="G61" s="13" t="n">
+        <x:v>-0.0053965403233687</x:v>
+      </x:c>
+      <x:c r="H61" s="12" t="n">
+        <x:v>-0.33848297872571487</x:v>
+      </x:c>
+      <x:c r="I61" s="11" t="n">
+        <x:v>-0.6527071129400469</x:v>
+      </x:c>
+      <x:c r="J61" s="11" t="n">
+        <x:v>1.0227692395126338</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="23" customHeight="1">
+      <x:c r="A62" s="2" t="str">
+        <x:v>THINK + mixer / Daily + AH + PM / seed 981756941</x:v>
+      </x:c>
+      <x:c r="B62" s="2" t="str">
+        <x:v>Individual-seed diagnostic</x:v>
+      </x:c>
+      <x:c r="C62" s="2" t="str">
+        <x:v>981756941</x:v>
+      </x:c>
+      <x:c r="D62" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E62" s="11" t="n">
+        <x:v>0.2932891759085201</x:v>
+      </x:c>
+      <x:c r="F62" s="12" t="n">
+        <x:v>0.07536932442510805</x:v>
+      </x:c>
+      <x:c r="G62" s="13" t="n">
+        <x:v>0.0064616708292001</x:v>
+      </x:c>
+      <x:c r="H62" s="12" t="n">
+        <x:v>-0.37603641351680805</x:v>
+      </x:c>
+      <x:c r="I62" s="11" t="n">
+        <x:v>-0.5925458391026873</x:v>
+      </x:c>
+      <x:c r="J62" s="11" t="n">
+        <x:v>1.1974231341327155</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="23" customHeight="1">
+      <x:c r="A63" s="2" t="str">
+        <x:v>SPY</x:v>
+      </x:c>
+      <x:c r="B63" s="2" t="str">
+        <x:v>Benchmark</x:v>
+      </x:c>
+      <x:c r="C63" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D63" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E63" s="11" t="n">
+        <x:v>0.49787510051856415</x:v>
+      </x:c>
+      <x:c r="F63" s="12" t="n">
+        <x:v>0.10852446279628823</x:v>
+      </x:c>
+      <x:c r="G63" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H63" s="12" t="n">
+        <x:v>-0.24550331508790435</x:v>
+      </x:c>
+      <x:c r="I63" s="11" t="n">
+        <x:v>-0.366633798605141</x:v>
+      </x:c>
+      <x:c r="J63" s="11" t="n">
+        <x:v>1.4189016899272882</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="23" customHeight="1">
+      <x:c r="A64" s="2" t="str">
+        <x:v>QQQ</x:v>
+      </x:c>
+      <x:c r="B64" s="2" t="str">
+        <x:v>Benchmark</x:v>
+      </x:c>
+      <x:c r="C64" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D64" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E64" s="11" t="n">
+        <x:v>0.46942259153465693</x:v>
+      </x:c>
+      <x:c r="F64" s="12" t="n">
+        <x:v>0.11931004741126919</x:v>
+      </x:c>
+      <x:c r="G64" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H64" s="12" t="n">
+        <x:v>-0.34874918657901777</x:v>
+      </x:c>
+      <x:c r="I64" s="11" t="n">
+        <x:v>-0.408298284123798</x:v>
+      </x:c>
+      <x:c r="J64" s="11" t="n">
+        <x:v>1.394466774653006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="23" customHeight="1">
+      <x:c r="A65" s="2" t="str">
+        <x:v>Monthly Nasdaq-100 basket</x:v>
+      </x:c>
+      <x:c r="B65" s="2" t="str">
+        <x:v>Benchmark</x:v>
+      </x:c>
+      <x:c r="C65" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D65" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E65" s="11" t="n">
+        <x:v>0.27856618099466113</x:v>
+      </x:c>
+      <x:c r="F65" s="12" t="n">
+        <x:v>0.06891999057407383</x:v>
+      </x:c>
+      <x:c r="G65" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H65" s="12" t="n">
+        <x:v>-0.30501562389730474</x:v>
+      </x:c>
+      <x:c r="I65" s="11" t="n">
+        <x:v>-0.5668889984851457</x:v>
+      </x:c>
+      <x:c r="J65" s="11" t="n">
+        <x:v>1.157622190839454</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="23" customHeight="1">
+      <x:c r="A66" s="2" t="str">
+        <x:v>SPY</x:v>
+      </x:c>
+      <x:c r="B66" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C66" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D66" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E66" s="11" t="n">
+        <x:v>0.4958585676015319</x:v>
+      </x:c>
+      <x:c r="F66" s="12" t="n">
+        <x:v>0.10812587715431944</x:v>
+      </x:c>
+      <x:c r="G66" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H66" s="12" t="n">
+        <x:v>-0.24604217502032333</x:v>
+      </x:c>
+      <x:c r="I66" s="11" t="n">
+        <x:v>-0.3678162983575254</x:v>
+      </x:c>
+      <x:c r="J66" s="11" t="n">
+        <x:v>1.416241125519769</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="23" customHeight="1">
+      <x:c r="A67" s="2" t="str">
+        <x:v>QQQ</x:v>
+      </x:c>
+      <x:c r="B67" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C67" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D67" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E67" s="11" t="n">
+        <x:v>0.46788215081819406</x:v>
+      </x:c>
+      <x:c r="F67" s="12" t="n">
+        <x:v>0.11890452555370727</x:v>
+      </x:c>
+      <x:c r="G67" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H67" s="12" t="n">
+        <x:v>-0.34921788093226946</x:v>
+      </x:c>
+      <x:c r="I67" s="11" t="n">
+        <x:v>-0.4101446435701171</x:v>
+      </x:c>
+      <x:c r="J67" s="11" t="n">
+        <x:v>1.3938072455646124</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="23" customHeight="1">
+      <x:c r="A68" s="2" t="str">
+        <x:v>Monthly Nasdaq-100 basket</x:v>
+      </x:c>
+      <x:c r="B68" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C68" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D68" s="29" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E68" s="11" t="n">
+        <x:v>0.27384401920831053</x:v>
+      </x:c>
+      <x:c r="F68" s="12" t="n">
+        <x:v>0.0678167340762789</x:v>
+      </x:c>
+      <x:c r="G68" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H68" s="12" t="n">
+        <x:v>-0.30586422964440463</x:v>
+      </x:c>
+      <x:c r="I68" s="11" t="n">
+        <x:v>-0.572165199807421</x:v>
+      </x:c>
+      <x:c r="J68" s="11" t="n">
+        <x:v>1.1540269210457577</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="23" customHeight="1">
+      <x:c r="A69" s="2" t="str">
+        <x:v>SPY</x:v>
+      </x:c>
+      <x:c r="B69" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C69" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D69" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E69" s="11" t="n">
+        <x:v>0.49181896886395904</x:v>
+      </x:c>
+      <x:c r="F69" s="12" t="n">
+        <x:v>0.10732914144148509</x:v>
+      </x:c>
+      <x:c r="G69" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H69" s="12" t="n">
+        <x:v>-0.24711758906306003</x:v>
+      </x:c>
+      <x:c r="I69" s="11" t="n">
+        <x:v>-0.3743372534563272</x:v>
+      </x:c>
+      <x:c r="J69" s="11" t="n">
+        <x:v>1.4129223556151047</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="23" customHeight="1">
+      <x:c r="A70" s="2" t="str">
+        <x:v>QQQ</x:v>
+      </x:c>
+      <x:c r="B70" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C70" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D70" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E70" s="11" t="n">
+        <x:v>0.4647985482573369</x:v>
+      </x:c>
+      <x:c r="F70" s="12" t="n">
+        <x:v>0.11809393168645213</x:v>
+      </x:c>
+      <x:c r="G70" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H70" s="12" t="n">
+        <x:v>-0.35015324867860276</x:v>
+      </x:c>
+      <x:c r="I70" s="11" t="n">
+        <x:v>-0.41231102061804</x:v>
+      </x:c>
+      <x:c r="J70" s="11" t="n">
+        <x:v>1.3930027543797971</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="23" customHeight="1">
+      <x:c r="A71" s="2" t="str">
+        <x:v>Monthly Nasdaq-100 basket</x:v>
+      </x:c>
+      <x:c r="B71" s="2" t="str">
+        <x:v>Cost sensitivity</x:v>
+      </x:c>
+      <x:c r="C71" s="2" t="str">
+        <x:v>ensemble</x:v>
+      </x:c>
+      <x:c r="D71" s="29" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E71" s="11" t="n">
+        <x:v>0.2644263109338815</x:v>
+      </x:c>
+      <x:c r="F71" s="12" t="n">
+        <x:v>0.06561939752700113</x:v>
+      </x:c>
+      <x:c r="G71" s="13" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="H71" s="12" t="n">
+        <x:v>-0.30754547996451354</x:v>
+      </x:c>
+      <x:c r="I71" s="11" t="n">
+        <x:v>-0.5819886420187742</x:v>
+      </x:c>
+      <x:c r="J71" s="11" t="n">
+        <x:v>1.1463717938073272</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9ff4ec99e40480a"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>